<commit_message>
Update MLB hitter fantasy scores 2026-08-03 (2026-08-02 08:17 PM)
</commit_message>
<xml_diff>
--- a/PRIZEPICKS_HITTER_AI_V5_TOP30_2026_08_03.xlsx
+++ b/PRIZEPICKS_HITTER_AI_V5_TOP30_2026_08_03.xlsx
@@ -4931,7 +4931,7 @@
         <v>287</v>
       </c>
       <c r="CL5" s="3" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="CM5" s="4" t="inlineStr">
         <is>
@@ -5783,7 +5783,7 @@
         <v>287</v>
       </c>
       <c r="CL6" s="3" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="CM6" s="4" t="inlineStr">
         <is>
@@ -10887,7 +10887,7 @@
         <v>287</v>
       </c>
       <c r="CL12" s="3" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="CM12" s="4" t="inlineStr">
         <is>
@@ -17679,7 +17679,7 @@
         <v>287</v>
       </c>
       <c r="CL20" s="3" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="CM20" s="4" t="inlineStr">
         <is>
@@ -19383,7 +19383,7 @@
         <v>287</v>
       </c>
       <c r="CL22" s="3" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="CM22" s="4" t="inlineStr">
         <is>
@@ -21923,7 +21923,7 @@
         <v>287</v>
       </c>
       <c r="CL25" s="3" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="CM25" s="4" t="inlineStr">
         <is>

</xml_diff>